<commit_message>
[feature]: codigo de modelamiento base
</commit_message>
<xml_diff>
--- a/documents/oferta_relevante.xlsx
+++ b/documents/oferta_relevante.xlsx
@@ -151,11 +151,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -633,13 +632,13 @@
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B26" s="3">
+      <c r="B26" s="1">
         <v>95</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="1" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>